<commit_message>
Updated Excel file - fixed formatting
</commit_message>
<xml_diff>
--- a/IT23332980_Assignment 1 - Test cases.xlsx
+++ b/IT23332980_Assignment 1 - Test cases.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sahan Mendis\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sahan Mendis\Desktop\IT23332980\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F8FB942-CEBE-4038-B544-2F2CFC63275D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35DFEF3D-4355-4D36-8C64-E86BCECE861E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,20 @@
     <sheet name="Test cases" sheetId="1" r:id="rId1"/>
     <sheet name="Coverage Summary" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -888,7 +901,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -897,6 +910,17 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -925,7 +949,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -939,6 +963,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -946,14 +980,16 @@
   <dxfs count="1">
     <dxf>
       <font>
-        <b/>
-        <color rgb="FFC00000"/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="0"/>
+        <name val="Carlito"/>
+        <scheme val="none"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FFFCE4D6"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -976,11 +1012,11 @@
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Input"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Expected output"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Actual output"/>
-    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Status"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Status" dataDxfId="0"/>
     <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="Singlish input types covered"/>
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="Evidence or rationale for the input type covered"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -1147,11 +1183,11 @@
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
-    <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="5" width="45" customWidth="1"/>
-    <col min="6" max="6" width="12" customWidth="1"/>
+    <col min="2" max="2" width="14.8984375" customWidth="1"/>
+    <col min="3" max="5" width="45.09765625" customWidth="1"/>
+    <col min="6" max="6" width="12" style="6" customWidth="1"/>
     <col min="7" max="7" width="32" customWidth="1"/>
-    <col min="8" max="8" width="65" customWidth="1"/>
+    <col min="8" max="8" width="101.3984375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="25.65" customHeight="1">
@@ -1170,7 +1206,7 @@
       <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
       <c r="G1" s="2" t="s">
@@ -1196,7 +1232,7 @@
       <c r="E2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="F2" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G2" s="3" t="s">
@@ -1222,7 +1258,7 @@
       <c r="E3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G3" s="3" t="s">
@@ -1248,7 +1284,7 @@
       <c r="E4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="F4" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G4" s="3" t="s">
@@ -1274,7 +1310,7 @@
       <c r="E5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="F5" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G5" s="3" t="s">
@@ -1300,7 +1336,7 @@
       <c r="E6" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G6" s="3" t="s">
@@ -1326,7 +1362,7 @@
       <c r="E7" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="F7" s="3" t="s">
+      <c r="F7" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G7" s="3" t="s">
@@ -1352,7 +1388,7 @@
       <c r="E8" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F8" s="3" t="s">
+      <c r="F8" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G8" s="3" t="s">
@@ -1378,7 +1414,7 @@
       <c r="E9" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="F9" s="3" t="s">
+      <c r="F9" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G9" s="3" t="s">
@@ -1404,7 +1440,7 @@
       <c r="E10" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="F10" s="3" t="s">
+      <c r="F10" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G10" s="3" t="s">
@@ -1430,7 +1466,7 @@
       <c r="E11" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="F11" s="3" t="s">
+      <c r="F11" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G11" s="3" t="s">
@@ -1456,7 +1492,7 @@
       <c r="E12" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="F12" s="3" t="s">
+      <c r="F12" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G12" s="3" t="s">
@@ -1482,7 +1518,7 @@
       <c r="E13" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="F13" s="3" t="s">
+      <c r="F13" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G13" s="3" t="s">
@@ -1508,7 +1544,7 @@
       <c r="E14" s="3" t="s">
         <v>79</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="F14" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G14" s="3" t="s">
@@ -1534,7 +1570,7 @@
       <c r="E15" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="F15" s="3" t="s">
+      <c r="F15" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G15" s="3" t="s">
@@ -1560,7 +1596,7 @@
       <c r="E16" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="F16" s="3" t="s">
+      <c r="F16" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G16" s="3" t="s">
@@ -1586,7 +1622,7 @@
       <c r="E17" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="F17" s="3" t="s">
+      <c r="F17" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G17" s="3" t="s">
@@ -1612,7 +1648,7 @@
       <c r="E18" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="F18" s="3" t="s">
+      <c r="F18" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G18" s="3" t="s">
@@ -1638,7 +1674,7 @@
       <c r="E19" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="F19" s="3" t="s">
+      <c r="F19" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G19" s="3" t="s">
@@ -1664,7 +1700,7 @@
       <c r="E20" s="3" t="s">
         <v>112</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="F20" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G20" s="3" t="s">
@@ -1690,7 +1726,7 @@
       <c r="E21" s="3" t="s">
         <v>118</v>
       </c>
-      <c r="F21" s="3" t="s">
+      <c r="F21" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G21" s="3" t="s">
@@ -1716,7 +1752,7 @@
       <c r="E22" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="F22" s="3" t="s">
+      <c r="F22" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G22" s="3" t="s">
@@ -1742,7 +1778,7 @@
       <c r="E23" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="F23" s="3" t="s">
+      <c r="F23" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G23" s="3" t="s">
@@ -1768,7 +1804,7 @@
       <c r="E24" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="F24" s="3" t="s">
+      <c r="F24" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G24" s="3" t="s">
@@ -1794,7 +1830,7 @@
       <c r="E25" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="F25" s="3" t="s">
+      <c r="F25" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G25" s="3" t="s">
@@ -1820,7 +1856,7 @@
       <c r="E26" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="F26" s="3" t="s">
+      <c r="F26" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G26" s="3" t="s">
@@ -1846,7 +1882,7 @@
       <c r="E27" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="F27" s="3" t="s">
+      <c r="F27" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G27" s="3" t="s">
@@ -1872,7 +1908,7 @@
       <c r="E28" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="F28" s="3" t="s">
+      <c r="F28" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G28" s="3" t="s">
@@ -1898,7 +1934,7 @@
       <c r="E29" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="F29" s="3" t="s">
+      <c r="F29" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G29" s="3" t="s">
@@ -1924,7 +1960,7 @@
       <c r="E30" s="3" t="s">
         <v>167</v>
       </c>
-      <c r="F30" s="3" t="s">
+      <c r="F30" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G30" s="3" t="s">
@@ -1950,7 +1986,7 @@
       <c r="E31" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="F31" s="3" t="s">
+      <c r="F31" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G31" s="3" t="s">
@@ -1976,7 +2012,7 @@
       <c r="E32" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="F32" s="3" t="s">
+      <c r="F32" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G32" s="3" t="s">
@@ -2002,7 +2038,7 @@
       <c r="E33" s="3" t="s">
         <v>184</v>
       </c>
-      <c r="F33" s="3" t="s">
+      <c r="F33" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G33" s="3" t="s">
@@ -2028,7 +2064,7 @@
       <c r="E34" s="3" t="s">
         <v>189</v>
       </c>
-      <c r="F34" s="3" t="s">
+      <c r="F34" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G34" s="3" t="s">
@@ -2054,7 +2090,7 @@
       <c r="E35" s="3" t="s">
         <v>195</v>
       </c>
-      <c r="F35" s="3" t="s">
+      <c r="F35" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G35" s="3" t="s">
@@ -2080,7 +2116,7 @@
       <c r="E36" s="3" t="s">
         <v>200</v>
       </c>
-      <c r="F36" s="3" t="s">
+      <c r="F36" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G36" s="3" t="s">
@@ -2106,7 +2142,7 @@
       <c r="E37" s="3" t="s">
         <v>206</v>
       </c>
-      <c r="F37" s="3" t="s">
+      <c r="F37" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G37" s="3" t="s">
@@ -2132,7 +2168,7 @@
       <c r="E38" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="F38" s="3" t="s">
+      <c r="F38" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G38" s="3" t="s">
@@ -2158,7 +2194,7 @@
       <c r="E39" s="3" t="s">
         <v>217</v>
       </c>
-      <c r="F39" s="3" t="s">
+      <c r="F39" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G39" s="3" t="s">
@@ -2184,7 +2220,7 @@
       <c r="E40" s="3" t="s">
         <v>222</v>
       </c>
-      <c r="F40" s="3" t="s">
+      <c r="F40" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G40" s="3" t="s">
@@ -2210,7 +2246,7 @@
       <c r="E41" s="3" t="s">
         <v>228</v>
       </c>
-      <c r="F41" s="3" t="s">
+      <c r="F41" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G41" s="3" t="s">
@@ -2236,7 +2272,7 @@
       <c r="E42" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="F42" s="3" t="s">
+      <c r="F42" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G42" s="3" t="s">
@@ -2262,7 +2298,7 @@
       <c r="E43" s="3" t="s">
         <v>239</v>
       </c>
-      <c r="F43" s="3" t="s">
+      <c r="F43" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G43" s="3" t="s">
@@ -2288,7 +2324,7 @@
       <c r="E44" s="3" t="s">
         <v>244</v>
       </c>
-      <c r="F44" s="3" t="s">
+      <c r="F44" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G44" s="3" t="s">
@@ -2314,7 +2350,7 @@
       <c r="E45" s="3" t="s">
         <v>250</v>
       </c>
-      <c r="F45" s="3" t="s">
+      <c r="F45" s="7" t="s">
         <v>13</v>
       </c>
       <c r="G45" s="3" t="s">
@@ -2340,7 +2376,7 @@
       <c r="E46" s="3" t="s">
         <v>255</v>
       </c>
-      <c r="F46" s="3" t="s">
+      <c r="F46" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G46" s="3" t="s">
@@ -2366,7 +2402,7 @@
       <c r="E47" s="3" t="s">
         <v>261</v>
       </c>
-      <c r="F47" s="3" t="s">
+      <c r="F47" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G47" s="3" t="s">
@@ -2392,7 +2428,7 @@
       <c r="E48" s="3" t="s">
         <v>266</v>
       </c>
-      <c r="F48" s="3" t="s">
+      <c r="F48" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G48" s="3" t="s">
@@ -2418,7 +2454,7 @@
       <c r="E49" s="3" t="s">
         <v>272</v>
       </c>
-      <c r="F49" s="3" t="s">
+      <c r="F49" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G49" s="3" t="s">
@@ -2444,7 +2480,7 @@
       <c r="E50" s="3" t="s">
         <v>277</v>
       </c>
-      <c r="F50" s="3" t="s">
+      <c r="F50" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G50" s="3" t="s">
@@ -2470,7 +2506,7 @@
       <c r="E51" s="3" t="s">
         <v>282</v>
       </c>
-      <c r="F51" s="3" t="s">
+      <c r="F51" s="8" t="s">
         <v>13</v>
       </c>
       <c r="G51" s="3" t="s">
@@ -2481,11 +2517,6 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F51">
-    <cfRule type="expression" dxfId="0" priority="1">
-      <formula>F2="FAIL"</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>

</xml_diff>